<commit_message>
Added Filter Data Table, Find even number from array, Group Function, Inner Join, Let Function, Order By LinQ, Remove Empty Rows,Sum Function
</commit_message>
<xml_diff>
--- a/InputFile/LetFuction.xlsx
+++ b/InputFile/LetFuction.xlsx
@@ -2,18 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RPA Project\LinQ\InputFile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{061EFCDE-847A-4CCC-B3C6-546CCF3E38FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50B13531-5B19-4383-AF2A-BF7A797645B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EEE198D2-21B0-42EA-BB53-967597C54CA3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{EEE198D2-21B0-42EA-BB53-967597C54CA3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="7" r:id="rId3"/>
+    <sheet name="Avearge" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="15">
   <si>
     <t>Id</t>
   </si>
@@ -36,6 +39,9 @@
     <t>Price</t>
   </si>
   <si>
+    <t>Count</t>
+  </si>
+  <si>
     <t>Milk</t>
   </si>
   <si>
@@ -54,7 +60,19 @@
     <t>Mango</t>
   </si>
   <si>
-    <t>Count</t>
+    <t>55</t>
+  </si>
+  <si>
+    <t>125</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>110</t>
   </si>
 </sst>
 </file>
@@ -420,7 +438,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -428,7 +446,7 @@
         <v>1452</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2">
         <v>55</v>
@@ -442,7 +460,7 @@
         <v>1452</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3">
         <v>40</v>
@@ -456,7 +474,7 @@
         <v>2541</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4">
         <v>125</v>
@@ -470,7 +488,7 @@
         <v>7412</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C5">
         <v>14</v>
@@ -484,7 +502,7 @@
         <v>8521</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C6">
         <v>55</v>
@@ -498,7 +516,7 @@
         <v>1235</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C7">
         <v>44</v>
@@ -512,7 +530,7 @@
         <v>1596</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C8">
         <v>110</v>
@@ -524,4 +542,404 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8171EACE-DF27-4C9E-BE27-F76E50227564}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1452</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>55</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2541</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>125</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>7412</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4">
+        <v>14</v>
+      </c>
+      <c r="D4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>8521</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>55</v>
+      </c>
+      <c r="D5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1235</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>44</v>
+      </c>
+      <c r="D6">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1596</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7">
+        <v>110</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4D8901E-1172-4EDF-8A34-B42EC12B8492}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1452</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>55</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2541</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>125</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>7412</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4">
+        <v>14</v>
+      </c>
+      <c r="D4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>8521</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>55</v>
+      </c>
+      <c r="D5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1235</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>44</v>
+      </c>
+      <c r="D6">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1596</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7">
+        <v>110</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>1452</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8">
+        <v>55</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>2541</v>
+      </c>
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9">
+        <v>125</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>7412</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10">
+        <v>14</v>
+      </c>
+      <c r="D10">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>8521</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11">
+        <v>55</v>
+      </c>
+      <c r="D11">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>1235</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12">
+        <v>44</v>
+      </c>
+      <c r="D12">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1596</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13">
+        <v>110</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>1452</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14">
+        <v>55</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1596</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15">
+        <v>110</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>8521</v>
+      </c>
+      <c r="B16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16">
+        <v>55</v>
+      </c>
+      <c r="D16">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+</worksheet>
 </file>
</xml_diff>